<commit_message>
update script and output files
average cost and gas sources shares
</commit_message>
<xml_diff>
--- a/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/costs_shares_IAEE_2025_run_2021.xlsx
+++ b/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/costs_shares_IAEE_2025_run_2021.xlsx
@@ -589,10 +589,10 @@
         <v>17504.28579187151</v>
       </c>
       <c r="C10" t="n">
-        <v>999999</v>
+        <v>6280.109140649178</v>
       </c>
       <c r="D10" t="n">
-        <v>1017503.285791871</v>
+        <v>23784.39493252068</v>
       </c>
     </row>
     <row r="11">
@@ -797,10 +797,10 @@
         <v>17862.49625626007</v>
       </c>
       <c r="C23" t="n">
-        <v>935089.2669528784</v>
+        <v>5585.361246760818</v>
       </c>
       <c r="D23" t="n">
-        <v>952951.7632091385</v>
+        <v>23447.85750302088</v>
       </c>
     </row>
     <row r="24">
@@ -845,7 +845,7 @@
         <v>14753.67547472048</v>
       </c>
       <c r="C26" t="n">
-        <v>7967.553166358784</v>
+        <v>7967.553166358783</v>
       </c>
       <c r="D26" t="n">
         <v>22721.22864107926</v>
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>23563.45671437721</v>
+        <v>23563.4567143772</v>
       </c>
       <c r="C29" t="n">
         <v>6721.87472281464</v>
@@ -1021,10 +1021,10 @@
         <v>17443.22340197671</v>
       </c>
       <c r="C37" t="n">
-        <v>48123.77669993664</v>
+        <v>3879.440191745927</v>
       </c>
       <c r="D37" t="n">
-        <v>65567.00010191335</v>
+        <v>21322.66359372264</v>
       </c>
     </row>
     <row r="38">
@@ -1101,10 +1101,10 @@
         <v>19750.49612200818</v>
       </c>
       <c r="C42" t="n">
-        <v>367028.8254690408</v>
+        <v>6248.183608719894</v>
       </c>
       <c r="D42" t="n">
-        <v>386779.321591049</v>
+        <v>25998.67973072807</v>
       </c>
     </row>
     <row r="43">
@@ -1245,7 +1245,7 @@
         <v>17832.48771802425</v>
       </c>
       <c r="C51" t="n">
-        <v>6030.183320704507</v>
+        <v>6030.183320704505</v>
       </c>
       <c r="D51" t="n">
         <v>23862.67103872876</v>
@@ -1309,10 +1309,10 @@
         <v>18774.60515931665</v>
       </c>
       <c r="C55" t="n">
-        <v>279068.7491917376</v>
+        <v>2133.232775926609</v>
       </c>
       <c r="D55" t="n">
-        <v>297843.3543510542</v>
+        <v>20907.83793524326</v>
       </c>
     </row>
     <row r="56">
@@ -2845,7 +2845,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.00207309164976824</v>
+        <v>0.002073091649768239</v>
       </c>
     </row>
     <row r="100">
@@ -2860,7 +2860,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>0.3082672931036552</v>
+        <v>0.3082672931036551</v>
       </c>
     </row>
     <row r="101">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>0.005557304716002368</v>
+        <v>0.005557304716002366</v>
       </c>
     </row>
     <row r="102">
@@ -2890,7 +2890,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>0.1393261653680574</v>
+        <v>0.1393261653680573</v>
       </c>
     </row>
     <row r="103">
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>0.04929495542312762</v>
+        <v>0.0492949554231276</v>
       </c>
     </row>
     <row r="105">
@@ -2950,7 +2950,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>0.004495667446859342</v>
+        <v>0.00449566744685934</v>
       </c>
     </row>
     <row r="107">
@@ -3040,7 +3040,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>0.05754573169201792</v>
+        <v>0.05754573169201791</v>
       </c>
     </row>
     <row r="113">
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>0.2784225690992297</v>
+        <v>0.2784225690992296</v>
       </c>
     </row>
     <row r="114">
@@ -3085,7 +3085,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>0.2703839391619798</v>
+        <v>0.2703839391619797</v>
       </c>
     </row>
     <row r="116">
@@ -4315,7 +4315,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>0.0008288425141636153</v>
+        <v>0.0008288425141636151</v>
       </c>
     </row>
     <row r="198">
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>0.00222186530600307</v>
+        <v>0.002221865306003069</v>
       </c>
     </row>
     <row r="202">
@@ -4390,7 +4390,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>0.05570397681421671</v>
+        <v>0.0557039768142167</v>
       </c>
     </row>
     <row r="203">

</xml_diff>